<commit_message>
Learn how to deploy website
</commit_message>
<xml_diff>
--- a/Week_10/Capstone Timesheet_Ripal Patel.xlsx
+++ b/Week_10/Capstone Timesheet_Ripal Patel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="109">
   <si>
     <t>Week_1</t>
   </si>
@@ -328,6 +328,31 @@
     <t>Search Best Hosting option to Deploy Website</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF000000"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t xml:space="preserve">Buy Domain (Godaddy) - </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF1155CC"/>
+        <sz val="12.0"/>
+        <u/>
+      </rPr>
+      <t>Healthcare-plus.info</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">check Video Tutorial For hosting - how to deploy PHP project + buy hosting from Hosinger </t>
+  </si>
+  <si>
+    <t>Production Testing (Services, Find a doctor page, services Page, Check Roles )</t>
+  </si>
+  <si>
     <t>Total Hours</t>
   </si>
 </sst>
@@ -339,7 +364,7 @@
     <numFmt numFmtId="164" formatCode="dd-mmm"/>
     <numFmt numFmtId="165" formatCode="d-mmm"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -392,6 +417,12 @@
       <sz val="11.0"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12.0"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="14.0"/>
@@ -504,7 +535,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="111">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -798,26 +829,21 @@
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    <xf borderId="1" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="10" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="10" fontId="10" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="10" fontId="11" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="10" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5687,9 +5713,15 @@
     </row>
     <row r="138">
       <c r="A138" s="102"/>
-      <c r="B138" s="101"/>
-      <c r="C138" s="103"/>
-      <c r="D138" s="100"/>
+      <c r="B138" s="103" t="s">
+        <v>105</v>
+      </c>
+      <c r="C138" s="99">
+        <v>46103.0</v>
+      </c>
+      <c r="D138" s="100">
+        <v>1.75</v>
+      </c>
       <c r="E138" s="3"/>
       <c r="F138" s="3"/>
       <c r="G138" s="3"/>
@@ -5716,9 +5748,15 @@
     </row>
     <row r="139">
       <c r="A139" s="102"/>
-      <c r="B139" s="101"/>
-      <c r="C139" s="103"/>
-      <c r="D139" s="100"/>
+      <c r="B139" s="101" t="s">
+        <v>106</v>
+      </c>
+      <c r="C139" s="99">
+        <v>46104.0</v>
+      </c>
+      <c r="D139" s="100">
+        <v>3.75</v>
+      </c>
       <c r="E139" s="3"/>
       <c r="F139" s="3"/>
       <c r="G139" s="3"/>
@@ -5744,10 +5782,16 @@
       <c r="AA139" s="3"/>
     </row>
     <row r="140">
-      <c r="A140" s="102"/>
-      <c r="B140" s="101"/>
-      <c r="C140" s="103"/>
-      <c r="D140" s="100"/>
+      <c r="A140" s="104"/>
+      <c r="B140" s="105" t="s">
+        <v>107</v>
+      </c>
+      <c r="C140" s="99">
+        <v>46104.0</v>
+      </c>
+      <c r="D140" s="105">
+        <v>2.15</v>
+      </c>
       <c r="E140" s="3"/>
       <c r="F140" s="3"/>
       <c r="G140" s="3"/>
@@ -5773,10 +5817,15 @@
       <c r="AA140" s="3"/>
     </row>
     <row r="141">
-      <c r="A141" s="104"/>
-      <c r="B141" s="105"/>
-      <c r="C141" s="99"/>
-      <c r="D141" s="106"/>
+      <c r="A141" s="102"/>
+      <c r="B141" s="106"/>
+      <c r="C141" s="107" t="s">
+        <v>15</v>
+      </c>
+      <c r="D141" s="106">
+        <f>(sum(D131:D140))</f>
+        <v>16.15</v>
+      </c>
       <c r="E141" s="3"/>
       <c r="F141" s="3"/>
       <c r="G141" s="3"/>
@@ -5802,10 +5851,10 @@
       <c r="AA141" s="3"/>
     </row>
     <row r="142">
-      <c r="A142" s="104"/>
-      <c r="B142" s="105"/>
-      <c r="C142" s="99"/>
-      <c r="D142" s="106"/>
+      <c r="A142" s="3"/>
+      <c r="B142" s="3"/>
+      <c r="C142" s="3"/>
+      <c r="D142" s="3"/>
       <c r="E142" s="3"/>
       <c r="F142" s="3"/>
       <c r="G142" s="3"/>
@@ -5831,10 +5880,10 @@
       <c r="AA142" s="3"/>
     </row>
     <row r="143">
-      <c r="A143" s="104"/>
-      <c r="B143" s="105"/>
-      <c r="C143" s="99"/>
-      <c r="D143" s="106"/>
+      <c r="A143" s="3"/>
+      <c r="B143" s="3"/>
+      <c r="C143" s="3"/>
+      <c r="D143" s="3"/>
       <c r="E143" s="3"/>
       <c r="F143" s="3"/>
       <c r="G143" s="3"/>
@@ -5860,10 +5909,10 @@
       <c r="AA143" s="3"/>
     </row>
     <row r="144">
-      <c r="A144" s="104"/>
-      <c r="B144" s="105"/>
-      <c r="C144" s="99"/>
-      <c r="D144" s="106"/>
+      <c r="A144" s="3"/>
+      <c r="B144" s="3"/>
+      <c r="C144" s="3"/>
+      <c r="D144" s="3"/>
       <c r="E144" s="3"/>
       <c r="F144" s="3"/>
       <c r="G144" s="3"/>
@@ -5889,10 +5938,15 @@
       <c r="AA144" s="3"/>
     </row>
     <row r="145">
-      <c r="A145" s="104"/>
-      <c r="B145" s="105"/>
-      <c r="C145" s="99"/>
-      <c r="D145" s="106"/>
+      <c r="A145" s="108" t="s">
+        <v>108</v>
+      </c>
+      <c r="B145" s="109"/>
+      <c r="C145" s="109"/>
+      <c r="D145" s="110">
+        <f>sum(D14,D34,D44,D54,D63,D73,D87,D105,D123)</f>
+        <v>169.1</v>
+      </c>
       <c r="E145" s="3"/>
       <c r="F145" s="3"/>
       <c r="G145" s="3"/>
@@ -5918,10 +5972,10 @@
       <c r="AA145" s="3"/>
     </row>
     <row r="146">
-      <c r="A146" s="102"/>
-      <c r="B146" s="105"/>
-      <c r="C146" s="99"/>
-      <c r="D146" s="106"/>
+      <c r="A146" s="3"/>
+      <c r="B146" s="3"/>
+      <c r="C146" s="3"/>
+      <c r="D146" s="3"/>
       <c r="E146" s="3"/>
       <c r="F146" s="3"/>
       <c r="G146" s="3"/>
@@ -5947,10 +6001,10 @@
       <c r="AA146" s="3"/>
     </row>
     <row r="147">
-      <c r="A147" s="102"/>
-      <c r="B147" s="105"/>
-      <c r="C147" s="99"/>
-      <c r="D147" s="106"/>
+      <c r="A147" s="3"/>
+      <c r="B147" s="3"/>
+      <c r="C147" s="3"/>
+      <c r="D147" s="3"/>
       <c r="E147" s="3"/>
       <c r="F147" s="3"/>
       <c r="G147" s="3"/>
@@ -5976,10 +6030,10 @@
       <c r="AA147" s="3"/>
     </row>
     <row r="148">
-      <c r="A148" s="107"/>
-      <c r="B148" s="107"/>
-      <c r="C148" s="107"/>
-      <c r="D148" s="107"/>
+      <c r="A148" s="3"/>
+      <c r="B148" s="3"/>
+      <c r="C148" s="3"/>
+      <c r="D148" s="3"/>
       <c r="E148" s="3"/>
       <c r="F148" s="3"/>
       <c r="G148" s="3"/>
@@ -6005,15 +6059,10 @@
       <c r="AA148" s="3"/>
     </row>
     <row r="149">
-      <c r="A149" s="102"/>
-      <c r="B149" s="102"/>
-      <c r="C149" s="108" t="s">
-        <v>15</v>
-      </c>
-      <c r="D149" s="102">
-        <f>(sum(D131:D147))</f>
-        <v>8.5</v>
-      </c>
+      <c r="A149" s="3"/>
+      <c r="B149" s="3"/>
+      <c r="C149" s="3"/>
+      <c r="D149" s="3"/>
       <c r="E149" s="3"/>
       <c r="F149" s="3"/>
       <c r="G149" s="3"/>
@@ -6126,15 +6175,10 @@
       <c r="AA152" s="3"/>
     </row>
     <row r="153">
-      <c r="A153" s="109" t="s">
-        <v>105</v>
-      </c>
-      <c r="B153" s="110"/>
-      <c r="C153" s="110"/>
-      <c r="D153" s="111">
-        <f>sum(D14,D34,D44,D54,D63,D73,D87,D105,D123)</f>
-        <v>169.1</v>
-      </c>
+      <c r="A153" s="3"/>
+      <c r="B153" s="3"/>
+      <c r="C153" s="3"/>
+      <c r="D153" s="3"/>
       <c r="E153" s="3"/>
       <c r="F153" s="3"/>
       <c r="G153" s="3"/>
@@ -30635,239 +30679,10 @@
       <c r="Z997" s="3"/>
       <c r="AA997" s="3"/>
     </row>
-    <row r="998">
-      <c r="A998" s="3"/>
-      <c r="B998" s="3"/>
-      <c r="C998" s="3"/>
-      <c r="D998" s="3"/>
-      <c r="E998" s="3"/>
-      <c r="F998" s="3"/>
-      <c r="G998" s="3"/>
-      <c r="H998" s="3"/>
-      <c r="I998" s="3"/>
-      <c r="J998" s="3"/>
-      <c r="K998" s="3"/>
-      <c r="L998" s="3"/>
-      <c r="M998" s="3"/>
-      <c r="N998" s="3"/>
-      <c r="O998" s="3"/>
-      <c r="P998" s="3"/>
-      <c r="Q998" s="3"/>
-      <c r="R998" s="3"/>
-      <c r="S998" s="3"/>
-      <c r="T998" s="3"/>
-      <c r="U998" s="3"/>
-      <c r="V998" s="3"/>
-      <c r="W998" s="3"/>
-      <c r="X998" s="3"/>
-      <c r="Y998" s="3"/>
-      <c r="Z998" s="3"/>
-      <c r="AA998" s="3"/>
-    </row>
-    <row r="999">
-      <c r="A999" s="3"/>
-      <c r="B999" s="3"/>
-      <c r="C999" s="3"/>
-      <c r="D999" s="3"/>
-      <c r="E999" s="3"/>
-      <c r="F999" s="3"/>
-      <c r="G999" s="3"/>
-      <c r="H999" s="3"/>
-      <c r="I999" s="3"/>
-      <c r="J999" s="3"/>
-      <c r="K999" s="3"/>
-      <c r="L999" s="3"/>
-      <c r="M999" s="3"/>
-      <c r="N999" s="3"/>
-      <c r="O999" s="3"/>
-      <c r="P999" s="3"/>
-      <c r="Q999" s="3"/>
-      <c r="R999" s="3"/>
-      <c r="S999" s="3"/>
-      <c r="T999" s="3"/>
-      <c r="U999" s="3"/>
-      <c r="V999" s="3"/>
-      <c r="W999" s="3"/>
-      <c r="X999" s="3"/>
-      <c r="Y999" s="3"/>
-      <c r="Z999" s="3"/>
-      <c r="AA999" s="3"/>
-    </row>
-    <row r="1000">
-      <c r="A1000" s="3"/>
-      <c r="B1000" s="3"/>
-      <c r="C1000" s="3"/>
-      <c r="D1000" s="3"/>
-      <c r="E1000" s="3"/>
-      <c r="F1000" s="3"/>
-      <c r="G1000" s="3"/>
-      <c r="H1000" s="3"/>
-      <c r="I1000" s="3"/>
-      <c r="J1000" s="3"/>
-      <c r="K1000" s="3"/>
-      <c r="L1000" s="3"/>
-      <c r="M1000" s="3"/>
-      <c r="N1000" s="3"/>
-      <c r="O1000" s="3"/>
-      <c r="P1000" s="3"/>
-      <c r="Q1000" s="3"/>
-      <c r="R1000" s="3"/>
-      <c r="S1000" s="3"/>
-      <c r="T1000" s="3"/>
-      <c r="U1000" s="3"/>
-      <c r="V1000" s="3"/>
-      <c r="W1000" s="3"/>
-      <c r="X1000" s="3"/>
-      <c r="Y1000" s="3"/>
-      <c r="Z1000" s="3"/>
-      <c r="AA1000" s="3"/>
-    </row>
-    <row r="1001">
-      <c r="A1001" s="3"/>
-      <c r="B1001" s="3"/>
-      <c r="C1001" s="3"/>
-      <c r="D1001" s="3"/>
-      <c r="E1001" s="3"/>
-      <c r="F1001" s="3"/>
-      <c r="G1001" s="3"/>
-      <c r="H1001" s="3"/>
-      <c r="I1001" s="3"/>
-      <c r="J1001" s="3"/>
-      <c r="K1001" s="3"/>
-      <c r="L1001" s="3"/>
-      <c r="M1001" s="3"/>
-      <c r="N1001" s="3"/>
-      <c r="O1001" s="3"/>
-      <c r="P1001" s="3"/>
-      <c r="Q1001" s="3"/>
-      <c r="R1001" s="3"/>
-      <c r="S1001" s="3"/>
-      <c r="T1001" s="3"/>
-      <c r="U1001" s="3"/>
-      <c r="V1001" s="3"/>
-      <c r="W1001" s="3"/>
-      <c r="X1001" s="3"/>
-      <c r="Y1001" s="3"/>
-      <c r="Z1001" s="3"/>
-      <c r="AA1001" s="3"/>
-    </row>
-    <row r="1002">
-      <c r="A1002" s="3"/>
-      <c r="B1002" s="3"/>
-      <c r="C1002" s="3"/>
-      <c r="D1002" s="3"/>
-      <c r="E1002" s="3"/>
-      <c r="F1002" s="3"/>
-      <c r="G1002" s="3"/>
-      <c r="H1002" s="3"/>
-      <c r="I1002" s="3"/>
-      <c r="J1002" s="3"/>
-      <c r="K1002" s="3"/>
-      <c r="L1002" s="3"/>
-      <c r="M1002" s="3"/>
-      <c r="N1002" s="3"/>
-      <c r="O1002" s="3"/>
-      <c r="P1002" s="3"/>
-      <c r="Q1002" s="3"/>
-      <c r="R1002" s="3"/>
-      <c r="S1002" s="3"/>
-      <c r="T1002" s="3"/>
-      <c r="U1002" s="3"/>
-      <c r="V1002" s="3"/>
-      <c r="W1002" s="3"/>
-      <c r="X1002" s="3"/>
-      <c r="Y1002" s="3"/>
-      <c r="Z1002" s="3"/>
-      <c r="AA1002" s="3"/>
-    </row>
-    <row r="1003">
-      <c r="A1003" s="3"/>
-      <c r="B1003" s="3"/>
-      <c r="C1003" s="3"/>
-      <c r="D1003" s="3"/>
-      <c r="E1003" s="3"/>
-      <c r="F1003" s="3"/>
-      <c r="G1003" s="3"/>
-      <c r="H1003" s="3"/>
-      <c r="I1003" s="3"/>
-      <c r="J1003" s="3"/>
-      <c r="K1003" s="3"/>
-      <c r="L1003" s="3"/>
-      <c r="M1003" s="3"/>
-      <c r="N1003" s="3"/>
-      <c r="O1003" s="3"/>
-      <c r="P1003" s="3"/>
-      <c r="Q1003" s="3"/>
-      <c r="R1003" s="3"/>
-      <c r="S1003" s="3"/>
-      <c r="T1003" s="3"/>
-      <c r="U1003" s="3"/>
-      <c r="V1003" s="3"/>
-      <c r="W1003" s="3"/>
-      <c r="X1003" s="3"/>
-      <c r="Y1003" s="3"/>
-      <c r="Z1003" s="3"/>
-      <c r="AA1003" s="3"/>
-    </row>
-    <row r="1004">
-      <c r="A1004" s="3"/>
-      <c r="B1004" s="3"/>
-      <c r="C1004" s="3"/>
-      <c r="D1004" s="3"/>
-      <c r="E1004" s="3"/>
-      <c r="F1004" s="3"/>
-      <c r="G1004" s="3"/>
-      <c r="H1004" s="3"/>
-      <c r="I1004" s="3"/>
-      <c r="J1004" s="3"/>
-      <c r="K1004" s="3"/>
-      <c r="L1004" s="3"/>
-      <c r="M1004" s="3"/>
-      <c r="N1004" s="3"/>
-      <c r="O1004" s="3"/>
-      <c r="P1004" s="3"/>
-      <c r="Q1004" s="3"/>
-      <c r="R1004" s="3"/>
-      <c r="S1004" s="3"/>
-      <c r="T1004" s="3"/>
-      <c r="U1004" s="3"/>
-      <c r="V1004" s="3"/>
-      <c r="W1004" s="3"/>
-      <c r="X1004" s="3"/>
-      <c r="Y1004" s="3"/>
-      <c r="Z1004" s="3"/>
-      <c r="AA1004" s="3"/>
-    </row>
-    <row r="1005">
-      <c r="A1005" s="3"/>
-      <c r="B1005" s="3"/>
-      <c r="C1005" s="3"/>
-      <c r="D1005" s="3"/>
-      <c r="E1005" s="3"/>
-      <c r="F1005" s="3"/>
-      <c r="G1005" s="3"/>
-      <c r="H1005" s="3"/>
-      <c r="I1005" s="3"/>
-      <c r="J1005" s="3"/>
-      <c r="K1005" s="3"/>
-      <c r="L1005" s="3"/>
-      <c r="M1005" s="3"/>
-      <c r="N1005" s="3"/>
-      <c r="O1005" s="3"/>
-      <c r="P1005" s="3"/>
-      <c r="Q1005" s="3"/>
-      <c r="R1005" s="3"/>
-      <c r="S1005" s="3"/>
-      <c r="T1005" s="3"/>
-      <c r="U1005" s="3"/>
-      <c r="V1005" s="3"/>
-      <c r="W1005" s="3"/>
-      <c r="X1005" s="3"/>
-      <c r="Y1005" s="3"/>
-      <c r="Z1005" s="3"/>
-      <c r="AA1005" s="3"/>
-    </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="B138"/>
+  </hyperlinks>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Manage-department and resolve conflicts
</commit_message>
<xml_diff>
--- a/Week_10/Capstone Timesheet_Ripal Patel.xlsx
+++ b/Week_10/Capstone Timesheet_Ripal Patel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="111">
   <si>
     <t>Week_1</t>
   </si>
@@ -328,29 +328,19 @@
     <t>Search Best Hosting option to Deploy Website</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF000000"/>
-        <sz val="12.0"/>
-      </rPr>
-      <t xml:space="preserve">Buy Domain (Godaddy) - </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <sz val="12.0"/>
-        <u/>
-      </rPr>
-      <t>Healthcare-plus.info</t>
-    </r>
+    <t>Buy Domain (Godaddy)</t>
   </si>
   <si>
     <t xml:space="preserve">check Video Tutorial For hosting - how to deploy PHP project + buy hosting from Hosinger </t>
   </si>
   <si>
     <t>Production Testing (Services, Find a doctor page, services Page, Check Roles )</t>
+  </si>
+  <si>
+    <t>Host Website resolve Errors</t>
+  </si>
+  <si>
+    <t>Update Manage Depatrment Conflicts + update admin panel + final Testing</t>
   </si>
   <si>
     <t>Total Hours</t>
@@ -364,7 +354,7 @@
     <numFmt numFmtId="164" formatCode="dd-mmm"/>
     <numFmt numFmtId="165" formatCode="d-mmm"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -417,12 +407,6 @@
       <sz val="11.0"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="12.0"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
     </font>
     <font>
       <sz val="14.0"/>
@@ -829,21 +813,21 @@
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="1" fillId="2" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="10" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="10" fontId="11" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="10" fontId="10" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="10" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5817,14 +5801,15 @@
       <c r="AA140" s="3"/>
     </row>
     <row r="141">
-      <c r="A141" s="102"/>
-      <c r="B141" s="106"/>
-      <c r="C141" s="107" t="s">
-        <v>15</v>
-      </c>
-      <c r="D141" s="106">
-        <f>(sum(D131:D140))</f>
-        <v>16.15</v>
+      <c r="A141" s="104"/>
+      <c r="B141" s="105" t="s">
+        <v>108</v>
+      </c>
+      <c r="C141" s="99">
+        <v>46106.0</v>
+      </c>
+      <c r="D141" s="105">
+        <v>1.75</v>
       </c>
       <c r="E141" s="3"/>
       <c r="F141" s="3"/>
@@ -5851,10 +5836,16 @@
       <c r="AA141" s="3"/>
     </row>
     <row r="142">
-      <c r="A142" s="3"/>
-      <c r="B142" s="3"/>
-      <c r="C142" s="3"/>
-      <c r="D142" s="3"/>
+      <c r="A142" s="104"/>
+      <c r="B142" s="105" t="s">
+        <v>109</v>
+      </c>
+      <c r="C142" s="99">
+        <v>46107.0</v>
+      </c>
+      <c r="D142" s="105">
+        <v>3.75</v>
+      </c>
       <c r="E142" s="3"/>
       <c r="F142" s="3"/>
       <c r="G142" s="3"/>
@@ -5880,10 +5871,15 @@
       <c r="AA142" s="3"/>
     </row>
     <row r="143">
-      <c r="A143" s="3"/>
-      <c r="B143" s="3"/>
-      <c r="C143" s="3"/>
-      <c r="D143" s="3"/>
+      <c r="A143" s="102"/>
+      <c r="B143" s="106"/>
+      <c r="C143" s="106" t="s">
+        <v>15</v>
+      </c>
+      <c r="D143" s="107">
+        <f>(sum(D131:D142))</f>
+        <v>21.65</v>
+      </c>
       <c r="E143" s="3"/>
       <c r="F143" s="3"/>
       <c r="G143" s="3"/>
@@ -5938,15 +5934,10 @@
       <c r="AA144" s="3"/>
     </row>
     <row r="145">
-      <c r="A145" s="108" t="s">
-        <v>108</v>
-      </c>
-      <c r="B145" s="109"/>
-      <c r="C145" s="109"/>
-      <c r="D145" s="110">
-        <f>sum(D14,D34,D44,D54,D63,D73,D87,D105,D123)</f>
-        <v>169.1</v>
-      </c>
+      <c r="A145" s="3"/>
+      <c r="B145" s="3"/>
+      <c r="C145" s="3"/>
+      <c r="D145" s="3"/>
       <c r="E145" s="3"/>
       <c r="F145" s="3"/>
       <c r="G145" s="3"/>
@@ -6001,10 +5992,15 @@
       <c r="AA146" s="3"/>
     </row>
     <row r="147">
-      <c r="A147" s="3"/>
-      <c r="B147" s="3"/>
-      <c r="C147" s="3"/>
-      <c r="D147" s="3"/>
+      <c r="A147" s="108" t="s">
+        <v>110</v>
+      </c>
+      <c r="B147" s="109"/>
+      <c r="C147" s="109"/>
+      <c r="D147" s="110">
+        <f>sum(D14,D34,D44,D54,D63,D73,D87,D105,D127,D143)</f>
+        <v>213</v>
+      </c>
       <c r="E147" s="3"/>
       <c r="F147" s="3"/>
       <c r="G147" s="3"/>
@@ -30679,10 +30675,65 @@
       <c r="Z997" s="3"/>
       <c r="AA997" s="3"/>
     </row>
+    <row r="998">
+      <c r="A998" s="3"/>
+      <c r="B998" s="3"/>
+      <c r="C998" s="3"/>
+      <c r="D998" s="3"/>
+      <c r="E998" s="3"/>
+      <c r="F998" s="3"/>
+      <c r="G998" s="3"/>
+      <c r="H998" s="3"/>
+      <c r="I998" s="3"/>
+      <c r="J998" s="3"/>
+      <c r="K998" s="3"/>
+      <c r="L998" s="3"/>
+      <c r="M998" s="3"/>
+      <c r="N998" s="3"/>
+      <c r="O998" s="3"/>
+      <c r="P998" s="3"/>
+      <c r="Q998" s="3"/>
+      <c r="R998" s="3"/>
+      <c r="S998" s="3"/>
+      <c r="T998" s="3"/>
+      <c r="U998" s="3"/>
+      <c r="V998" s="3"/>
+      <c r="W998" s="3"/>
+      <c r="X998" s="3"/>
+      <c r="Y998" s="3"/>
+      <c r="Z998" s="3"/>
+      <c r="AA998" s="3"/>
+    </row>
+    <row r="999">
+      <c r="A999" s="3"/>
+      <c r="B999" s="3"/>
+      <c r="C999" s="3"/>
+      <c r="D999" s="3"/>
+      <c r="E999" s="3"/>
+      <c r="F999" s="3"/>
+      <c r="G999" s="3"/>
+      <c r="H999" s="3"/>
+      <c r="I999" s="3"/>
+      <c r="J999" s="3"/>
+      <c r="K999" s="3"/>
+      <c r="L999" s="3"/>
+      <c r="M999" s="3"/>
+      <c r="N999" s="3"/>
+      <c r="O999" s="3"/>
+      <c r="P999" s="3"/>
+      <c r="Q999" s="3"/>
+      <c r="R999" s="3"/>
+      <c r="S999" s="3"/>
+      <c r="T999" s="3"/>
+      <c r="U999" s="3"/>
+      <c r="V999" s="3"/>
+      <c r="W999" s="3"/>
+      <c r="X999" s="3"/>
+      <c r="Y999" s="3"/>
+      <c r="Z999" s="3"/>
+      <c r="AA999" s="3"/>
+    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink r:id="rId1" ref="B138"/>
-  </hyperlinks>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>